<commit_message>
[Setting] 도감 UI 틀 만들기
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/DNItem.xlsx
+++ b/JsonConverter/ExcelFiles/DNItem.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fileVersion appName="HCell" lastEdited="12.0" lowestEdited="12.0" rupBuild="0.535"/>
+  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12458"/>
   <x:workbookPr date1904="0" showBorderUnselectedTables="1" filterPrivacy="0" promptedSolutions="0" showInkAnnotation="1" backupFile="0" saveExternalLinkValues="1" codeName="ThisWorkbook" hidePivotFieldList="0" allowRefreshQuery="0" publishItems="0" checkCompatibility="0" autoCompressPictures="1" refreshAllConnections="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_NRUnityProjects\UnityBasic_6\JsonConverter\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_NRUnityProjects\2DMainProject\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="4294934950" windowHeight="6150"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="22788" windowHeight="8520"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -21,6 +21,105 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
   <x:si>
+    <x:t>Icon/Icon_Item_Box_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_Gold_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_DummyBox_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>착용하면 공격력이 강해진다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SellingPrice</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Potato_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxStackCount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>지역에 나타나는 금화</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Corn_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Gold_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Equipment</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ItemType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>옥수수다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Normal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Legend</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Epic</x:t>
+  </x:si>
+  <x:si>
+    <x:t>의문의 모자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>옥수수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>화폐</x:t>
+  </x:si>
+  <x:si>
+    <x:t>감자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_Equip_Hat_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>감자다. 딱히 의미가 있진 않다.</x:t>
+  </x:si>
+  <x:si>
     <x:t>Item_Equip_Hat_1</x:t>
   </x:si>
   <x:si>
@@ -28,105 +127,6 @@
   </x:si>
   <x:si>
     <x:t>상자다. 딱히 의미가 있진 않다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>옥수수다</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Grade</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Epic</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Legend</x:t>
-  </x:si>
-  <x:si>
-    <x:t>의문의 모자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Normal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Equipment</x:t>
-  </x:si>
-  <x:si>
-    <x:t>지역에 나타나는 금화</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ItemType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SellingPrice</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_DummyBox_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxStackCount</x:t>
-  </x:si>
-  <x:si>
-    <x:t>착용하면 공격력이 강해진다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Gold_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Corn_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>상자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>옥수수</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>화폐</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Potato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Box_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Gold_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Equip_Hat_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>감자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>감자다. 딱히 의미가 있진 않다.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -228,16 +228,16 @@
   <x:borders count="2">
     <x:border>
       <x:left>
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
       </x:left>
       <x:right>
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
       </x:right>
       <x:top>
         <x:color auto="1"/>
       </x:top>
       <x:bottom>
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
       </x:bottom>
     </x:border>
     <x:border>
@@ -261,8 +261,8 @@
     </x:xf>
   </x:cellStyleXfs>
   <x:cellXfs count="16">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
@@ -319,6 +319,7 @@
         <x:dxf hs:applyExtension="1">
           <x:font hs:extension="1">
             <x:color rgb="ff000000"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -401,6 +402,7 @@
           <x:font hs:extension="1">
             <x:color rgb="ffffffff"/>
             <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -435,6 +437,7 @@
           <x:font hs:extension="1">
             <x:color rgb="ffffffff"/>
             <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -479,6 +482,7 @@
           <x:font hs:extension="1">
             <x:color rgb="ffffffff"/>
             <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -522,6 +526,7 @@
         <x:dxf hs:applyExtension="1">
           <x:font hs:extension="1">
             <x:color rgb="ff000000"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -606,6 +611,7 @@
         <x:dxf hs:applyExtension="1">
           <x:font hs:extension="1">
             <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -626,6 +632,7 @@
         <x:dxf hs:applyExtension="1">
           <x:font hs:extension="1">
             <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -656,6 +663,7 @@
         <x:dxf hs:applyExtension="1">
           <x:font hs:extension="1">
             <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
             <hs:size val="0"/>
             <hs:ratio val="0"/>
             <hs:spacing val="0"/>
@@ -904,9 +912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetPr codeName="Sheet1">
-    <x:outlinePr applyStyles="0" summaryBelow="0" summaryRight="1" showOutlineSymbols="1"/>
-  </x:sheetPr>
+  <x:sheetPr codeName="Sheet1"/>
   <x:dimension ref="A1:M35"/>
   <x:sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
@@ -921,80 +927,80 @@
   <x:sheetData>
     <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:8" ht="13.199999999999999">
+      <x:c r="A2" s="1" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
         <x:v>19</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:8" ht="13.19999999999999928946">
-      <x:c r="A2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8" s="12" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="11" t="s">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B3" s="11" t="s">
-        <x:v>6</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C3" s="11" t="s">
-        <x:v>23</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E3" s="13" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="F3" s="13" t="s">
-        <x:v>17</x:v>
-      </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H3" s="13" t="s">
-        <x:v>24</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>2</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E4" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F4" s="4">
         <x:v>20</x:v>
@@ -1003,7 +1009,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="H4" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="4"/>
       <x:c r="J4" s="4"/>
@@ -1013,19 +1019,19 @@
     </x:row>
     <x:row r="5" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>13</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
-        <x:v>9</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F5" s="4">
         <x:v>1000</x:v>
@@ -1034,7 +1040,7 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="H5" s="4" t="s">
-        <x:v>32</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="4"/>
       <x:c r="J5" s="4"/>
@@ -1044,19 +1050,19 @@
     </x:row>
     <x:row r="6" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>0</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>10</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E6" s="4" t="s">
-        <x:v>8</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F6" s="4">
         <x:v>0</x:v>
@@ -1065,7 +1071,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H6" s="4" t="s">
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="I6" s="4"/>
       <x:c r="K6" s="4"/>
@@ -1074,19 +1080,19 @@
     </x:row>
     <x:row r="7" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>22</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>4</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E7" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F7" s="4">
         <x:v>100</x:v>
@@ -1095,7 +1101,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="H7" s="4" t="s">
-        <x:v>1</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
@@ -1105,19 +1111,19 @@
     </x:row>
     <x:row r="8" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A8" s="15" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>34</x:v>
-      </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>35</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E8" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F8" s="4">
         <x:v>20</x:v>
@@ -1126,7 +1132,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="H8" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="4"/>
       <x:c r="J8" s="4"/>
@@ -2305,7 +2311,7 @@
     <x:row r="999" ht="15.75" customHeight="1"/>
     <x:row r="1000" ht="15.75" customHeight="1"/>
   </x:sheetData>
-  <x:pageMargins left="0.69986110925674438477" right="0.69986110925674438477" top="0.75" bottom="0.75" header="0.30000001192092895508" footer="0.30000001192092895508"/>
+  <x:pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="600" verticalDpi="600" copies="1"/>
 </x:worksheet>
 </file>
</xml_diff>